<commit_message>
Add 'Top level' column to release pool for backfill targeting
build_excel: hitter and pitcher Release_Pool sheets gain a 'Top level'
column showing the highest level each overflow player would project to
if a slot were available. Hitter ceiling = woba_max_level (with the
PREMIUM_WOBA_RELAX rule applied); pitcher ceiling = the more
restrictive of pwoba_top_level and age_top_level_pitcher (mirrors how
build_pitcher_system computes _top). Two new helpers in build_excel
(_hitter_top_level / _pitcher_top_level) so streamlit_app can reuse
the same logic.

streamlit_app: new 'Release pool' tab beside Overview / Rosters by level.
Two-column layout — hitters on the left (sorted by BestP desc), pitchers
on the right (sorted by rp_warP desc). Each row shows Top level so users
can spot which gaps each release candidate would slot into when manually
backfilling expanded minor-league rosters.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/LAA_roster_system.xlsx
+++ b/outputs/LAA_roster_system.xlsx
@@ -4013,7 +4013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4021,6 +4021,7 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -4048,10 +4049,15 @@
       </c>
       <c r="D3" s="32" t="inlineStr">
         <is>
+          <t>Top level</t>
+        </is>
+      </c>
+      <c r="E3" s="32" t="inlineStr">
+        <is>
           <t>Best</t>
         </is>
       </c>
-      <c r="E3" s="32" t="inlineStr">
+      <c r="F3" s="32" t="inlineStr">
         <is>
           <t>BestP</t>
         </is>
@@ -4071,10 +4077,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>-0.5</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="F4" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -4092,10 +4103,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>-2.1</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>1.3</v>
       </c>
     </row>
@@ -4113,10 +4129,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>-3.7</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>1.1</v>
       </c>
     </row>
@@ -4134,10 +4155,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>-2</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>0.8</v>
       </c>
     </row>
@@ -4155,10 +4181,15 @@
           <t>CF</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>-4.3</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -4176,10 +4207,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>-3.9</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -4197,10 +4233,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
         <v>-8.5</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -4218,10 +4259,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
         <v>-3.5</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -4239,10 +4285,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>-5.1</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>-1.3</v>
       </c>
     </row>
@@ -4260,10 +4311,15 @@
           <t>DH</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
         <v>-4.8</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>-1.3</v>
       </c>
     </row>
@@ -4281,10 +4337,15 @@
           <t>3B</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>-5.5</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>-1.5</v>
       </c>
     </row>
@@ -4302,10 +4363,15 @@
           <t>1B</t>
         </is>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
         <v>-6.5</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>-1.6</v>
       </c>
     </row>
@@ -4323,10 +4389,15 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
         <v>-3.7</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="F16" s="4" t="n">
         <v>-1.6</v>
       </c>
     </row>
@@ -4344,10 +4415,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
         <v>-8.199999999999999</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>-1.7</v>
       </c>
     </row>
@@ -4365,10 +4441,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
         <v>-9.199999999999999</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="F18" s="4" t="n">
         <v>-1.8</v>
       </c>
     </row>
@@ -4386,10 +4467,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
         <v>-6.8</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="F19" s="4" t="n">
         <v>-1.9</v>
       </c>
     </row>
@@ -4407,10 +4493,15 @@
           <t>3B</t>
         </is>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n">
         <v>-4.8</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="F20" s="4" t="n">
         <v>-2.1</v>
       </c>
     </row>
@@ -4428,10 +4519,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D21" s="4" t="n">
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n">
         <v>-6.8</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="F21" s="4" t="n">
         <v>-2.1</v>
       </c>
     </row>
@@ -4449,10 +4545,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D22" s="4" t="n">
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
         <v>-6.5</v>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="F22" s="4" t="n">
         <v>-2.1</v>
       </c>
     </row>
@@ -4470,10 +4571,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
         <v>-4.8</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="F23" s="4" t="n">
         <v>-2.2</v>
       </c>
     </row>
@@ -4491,10 +4597,15 @@
           <t>1B</t>
         </is>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
         <v>-4.4</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="F24" s="4" t="n">
         <v>-2.2</v>
       </c>
     </row>
@@ -4512,10 +4623,15 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
         <v>-5.5</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="F25" s="4" t="n">
         <v>-2.3</v>
       </c>
     </row>
@@ -4533,10 +4649,15 @@
           <t>1B</t>
         </is>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
         <v>-7</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="F26" s="4" t="n">
         <v>-2.5</v>
       </c>
     </row>
@@ -4554,10 +4675,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
         <v>-11.1</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="F27" s="4" t="n">
         <v>-2.5</v>
       </c>
     </row>
@@ -4575,10 +4701,15 @@
           <t>RF</t>
         </is>
       </c>
-      <c r="D28" s="4" t="n">
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
         <v>-5.4</v>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="F28" s="4" t="n">
         <v>-2.6</v>
       </c>
     </row>
@@ -4596,10 +4727,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
         <v>-5.1</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="F29" s="4" t="n">
         <v>-3</v>
       </c>
     </row>
@@ -4617,10 +4753,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D30" s="4" t="n">
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
         <v>-4.3</v>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="F30" s="4" t="n">
         <v>-3.3</v>
       </c>
     </row>
@@ -4638,10 +4779,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="n">
         <v>-7.4</v>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="F31" s="4" t="n">
         <v>-3.5</v>
       </c>
     </row>
@@ -4659,10 +4805,15 @@
           <t>1B</t>
         </is>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
         <v>-11.8</v>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="F32" s="4" t="n">
         <v>-3.9</v>
       </c>
     </row>
@@ -4680,10 +4831,15 @@
           <t>1B</t>
         </is>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
         <v>-7.5</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="F33" s="4" t="n">
         <v>-4.1</v>
       </c>
     </row>
@@ -4701,10 +4857,15 @@
           <t>SS</t>
         </is>
       </c>
-      <c r="D34" s="4" t="n">
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
         <v>-8.800000000000001</v>
       </c>
-      <c r="E34" s="4" t="n">
+      <c r="F34" s="4" t="n">
         <v>-4.3</v>
       </c>
     </row>
@@ -4722,10 +4883,15 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
         <v>-11.2</v>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="F35" s="4" t="n">
         <v>-4.4</v>
       </c>
     </row>
@@ -4743,10 +4909,15 @@
           <t>1B</t>
         </is>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="n">
         <v>-8.9</v>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="F36" s="4" t="n">
         <v>-5.1</v>
       </c>
     </row>
@@ -4764,10 +4935,15 @@
           <t>2B</t>
         </is>
       </c>
-      <c r="D37" s="4" t="n">
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="n">
         <v>-10.5</v>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="F37" s="4" t="n">
         <v>-5.2</v>
       </c>
     </row>
@@ -4785,10 +4961,15 @@
           <t>3B</t>
         </is>
       </c>
-      <c r="D38" s="4" t="n">
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
         <v>-13.3</v>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="F38" s="4" t="n">
         <v>-6.2</v>
       </c>
     </row>
@@ -4806,10 +4987,15 @@
           <t>1B</t>
         </is>
       </c>
-      <c r="D39" s="4" t="n">
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>R(DLR)</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n">
         <v>-12.3</v>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="F39" s="4" t="n">
         <v>-6.4</v>
       </c>
     </row>
@@ -4827,16 +5013,21 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D40" s="4" t="n">
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
         <v>-6.7</v>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="F40" s="4" t="n">
         <v>-6.4</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4848,15 +5039,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -4879,20 +5071,25 @@
       </c>
       <c r="C3" s="32" t="inlineStr">
         <is>
+          <t>Top level</t>
+        </is>
+      </c>
+      <c r="D3" s="32" t="inlineStr">
+        <is>
           <t>pwOBA</t>
         </is>
       </c>
-      <c r="D3" s="32" t="inlineStr">
+      <c r="E3" s="32" t="inlineStr">
         <is>
           <t>sp_warP</t>
         </is>
       </c>
-      <c r="E3" s="32" t="inlineStr">
+      <c r="F3" s="32" t="inlineStr">
         <is>
           <t>rp_warP</t>
         </is>
       </c>
-      <c r="F3" s="32" t="inlineStr">
+      <c r="G3" s="32" t="inlineStr">
         <is>
           <t>IP</t>
         </is>
@@ -4907,14 +5104,19 @@
       <c r="B4" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>0.403</v>
       </c>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="n">
         <v>-0.6</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="G4" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4927,16 +5129,21 @@
       <c r="B5" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>0.395</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>-2</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>-0.7</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4949,14 +5156,19 @@
       <c r="B6" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>0.403</v>
       </c>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="n">
         <v>-0.7</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="G6" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4969,14 +5181,19 @@
       <c r="B7" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>0.388</v>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="n">
         <v>-0.8</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="G7" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4989,16 +5206,21 @@
       <c r="B8" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>-2.4</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>-0.8</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5011,14 +5233,19 @@
       <c r="B9" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
         <v>0.403</v>
       </c>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="n">
         <v>-1</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5031,16 +5258,21 @@
       <c r="B10" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
         <v>0.401</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="E10" s="4" t="n">
         <v>-3</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>-1</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="G10" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5053,16 +5285,21 @@
       <c r="B11" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
         <v>0.396</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E11" s="4" t="n">
         <v>-3.4</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>-1.1</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5075,16 +5312,21 @@
       <c r="B12" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
         <v>0.402</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>-3.3</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>-1.1</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5097,16 +5339,21 @@
       <c r="B13" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
         <v>0.403</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="E13" s="4" t="n">
         <v>-3.6</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>-1.2</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="G13" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5119,16 +5366,21 @@
       <c r="B14" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>-3.5</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>-1.2</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5141,16 +5393,21 @@
       <c r="B15" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
         <v>0.402</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="E15" s="4" t="n">
         <v>-4</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>-1.3</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="G15" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5163,14 +5420,19 @@
       <c r="B16" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
         <v>0.396</v>
       </c>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="n">
         <v>-1.4</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5183,16 +5445,21 @@
       <c r="B17" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
         <v>0.395</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="E17" s="4" t="n">
         <v>-4.2</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>-1.4</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5205,14 +5472,19 @@
       <c r="B18" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="n">
         <v>-1.4</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="G18" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5225,22 +5497,27 @@
       <c r="B19" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
         <v>0.4</v>
       </c>
-      <c r="D19" s="4" t="n">
+      <c r="E19" s="4" t="n">
         <v>-4.2</v>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="F19" s="4" t="n">
         <v>-1.4</v>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="G19" s="4" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lower MINIMUM_RELIEVER_PITCHES from 2 to 1
A 1-pitch reliever is a real role — sidearm sinker specialists, ROOGY/
LOOGY types whose MLB value is one elite pitch (Ryan Thompson on AZ:
stuff 45/35, hra 65/45, ctrl 65/55 → only one pitch type above
PITCH_MINIMUM_RATING but a viable RHP specialist). At threshold 2 they
were tagged sprp='', got NaN pwOBAP, and the EXPORT_PAGES pwOBAP < 1.000
filter dropped them entirely from pitchers.json. Lowering to 1 admits
them; their pwOBA naturally places them at the right level (Thompson:
.315 → MLB-eligible, sp_warP None, rp_warP near-zero, lands as MLB RP).

Adds ~1,200 1-pitch arms to the pool — mostly minor-league depth where
the pool was thin anyway. 69 of them are MLB-quality (pwOBA ≤ .345).

LAA catcher placements unchanged.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/LAA_roster_system.xlsx
+++ b/outputs/LAA_roster_system.xlsx
@@ -1090,27 +1090,27 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Liam Peterson</t>
+          <t>Walbert Urena</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.369</v>
+        <v>0.334</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.3</v>
+        <v>0.312</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Mid-rotation</t>
+          <t>Back-end starter</t>
         </is>
       </c>
     </row>
@@ -1122,20 +1122,20 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Brody Hopkins</t>
+          <t>Liam Peterson</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.339</v>
+        <v>0.369</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.309</v>
+        <v>0.3</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.6</v>
+        <v>1.2</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0</v>
@@ -1154,27 +1154,27 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Victor Mederos</t>
+          <t>Brody Hopkins</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
         <v>25</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.354</v>
+        <v>0.339</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.331</v>
+        <v>0.309</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>-0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Innings eater</t>
+          <t>Mid-rotation</t>
         </is>
       </c>
     </row>
@@ -1186,23 +1186,23 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Braxton Bragg</t>
+          <t>Victor Mederos</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.356</v>
+        <v>0.354</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.33</v>
+        <v>0.331</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>-0.7</v>
+        <v>-0.8</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
@@ -1218,23 +1218,23 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Caden Dana</t>
+          <t>Braxton Bragg</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.364</v>
+        <v>0.356</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.336</v>
+        <v>0.33</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>-1.1</v>
+        <v>-0.7</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -1417,20 +1417,20 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Carlos Espinosa</t>
+          <t>Jose Gonzalez</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
         <v>25</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.38</v>
+        <v>0.373</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.322</v>
+        <v>0.355</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>-0.1</v>
+        <v>-0.8</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>0</v>
@@ -1449,27 +1449,27 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Bridger Holmes</t>
+          <t>Carlos Espinosa</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.382</v>
+        <v>0.38</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.32</v>
+        <v>0.322</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Mid leverage</t>
+          <t>Low leverage / depth</t>
         </is>
       </c>
     </row>
@@ -1481,27 +1481,27 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Lucas Mahlstedt</t>
+          <t>Bridger Holmes</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
         <v>24</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.384</v>
+        <v>0.382</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.323</v>
+        <v>0.32</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>-0.1</v>
+        <v>-0</v>
       </c>
       <c r="G18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Low leverage / depth</t>
+          <t>Mid leverage</t>
         </is>
       </c>
     </row>
@@ -1605,17 +1605,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Franklin Gomez</t>
+          <t>Caden Dana</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.376</v>
+        <v>0.364</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.335</v>
+        <v>0.336</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>-1.1</v>
@@ -1637,27 +1637,27 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Tyler Bremner</t>
+          <t>Franklin Gomez</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.375</v>
+        <v>0.376</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.318</v>
+        <v>0.335</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.1</v>
+        <v>-1.1</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Back-end starter</t>
+          <t>Innings eater</t>
         </is>
       </c>
     </row>
@@ -1669,27 +1669,27 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Joel Hurtado</t>
+          <t>Tyler Bremner</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.366</v>
+        <v>0.375</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.328</v>
+        <v>0.318</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>-0.6</v>
+        <v>0.1</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Innings eater</t>
+          <t>Back-end starter</t>
         </is>
       </c>
     </row>
@@ -1701,27 +1701,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Austin Gordon</t>
+          <t>Joel Hurtado</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.383</v>
+        <v>0.366</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.314</v>
+        <v>0.328</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.3</v>
+        <v>-0.6</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Back-end starter</t>
+          <t>Innings eater</t>
         </is>
       </c>
     </row>
@@ -1733,27 +1733,27 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Jose Gonzalez</t>
+          <t>Austin Gordon</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.373</v>
+        <v>0.383</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.355</v>
+        <v>0.314</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>-2.4</v>
+        <v>0.3</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Innings eater</t>
+          <t>Back-end starter</t>
         </is>
       </c>
     </row>
@@ -1868,20 +1868,20 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Samy Natera Jr.</t>
+          <t>Lucas Mahlstedt</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.379</v>
+        <v>0.384</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.372</v>
+        <v>0.323</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>-1.2</v>
+        <v>-0.1</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>0</v>
@@ -1900,20 +1900,20 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Fulton Lockhart</t>
+          <t>Samy Natera Jr.</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.393</v>
+        <v>0.379</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.345</v>
+        <v>0.372</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>-0.6</v>
+        <v>-1.2</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>0</v>
@@ -1932,20 +1932,20 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Yeferson Vargas</t>
+          <t>Fulton Lockhart</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.394</v>
+        <v>0.393</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.354</v>
+        <v>0.345</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>-0.8</v>
+        <v>-0.6</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>0</v>
@@ -1964,17 +1964,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Owen Wild</t>
+          <t>Yeferson Vargas</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.385</v>
+        <v>0.394</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.357</v>
+        <v>0.354</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>-0.8</v>
@@ -1996,20 +1996,20 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Peyton Olejnik</t>
+          <t>Efrain Contreras</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.389</v>
+        <v>0.384</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.35</v>
+        <v>0.383</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>-0.7</v>
+        <v>-1.4</v>
       </c>
       <c r="G18" s="4" t="n">
         <v>0</v>
@@ -2383,20 +2383,20 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Freddy Hernandez</t>
+          <t>Jhon Almonte</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.4</v>
+        <v>0.403</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.374</v>
+        <v>0.357</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>-1.2</v>
+        <v>-0.8</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>0</v>
@@ -2415,17 +2415,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Luke Schmolke</t>
+          <t>Owen Wild</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.395</v>
+        <v>0.385</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.354</v>
+        <v>0.357</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>-0.8</v>
@@ -2447,20 +2447,20 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Tate McKee</t>
+          <t>Peyton Olejnik</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.403</v>
+        <v>0.389</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>-0.5</v>
+        <v>-0.7</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>0</v>
@@ -2834,20 +2834,20 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Fabian Soto</t>
+          <t>Freddy Hernandez</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>0.4</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0.368</v>
+        <v>0.374</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>-1.1</v>
+        <v>-1.2</v>
       </c>
       <c r="G12" s="4" t="n">
         <v>0</v>
@@ -2866,20 +2866,20 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Juan Jordan</t>
+          <t>Luke Schmolke</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.402</v>
+        <v>0.395</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.377</v>
+        <v>0.354</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>-1.3</v>
+        <v>-0.8</v>
       </c>
       <c r="G13" s="4" t="n">
         <v>0</v>
@@ -2898,20 +2898,20 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Cole Raymond</t>
+          <t>Tate McKee</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.401</v>
+        <v>0.403</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.369</v>
+        <v>0.34</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>-1.1</v>
+        <v>-0.5</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>0</v>
@@ -2930,20 +2930,20 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Jhostin Betances</t>
+          <t>Fabian Soto</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>0.4</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.373</v>
+        <v>0.368</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>-1.2</v>
+        <v>-1.1</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>0</v>
@@ -2962,17 +2962,17 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Sebastian Caseres</t>
+          <t>Juan Jordan</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
         <v>19</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.401</v>
+        <v>0.402</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.381</v>
+        <v>0.377</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>-1.3</v>
@@ -2994,20 +2994,20 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Anllelo Gutierrez</t>
+          <t>Cole Raymond</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>0.403</v>
+        <v>0.401</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.381</v>
+        <v>0.369</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>-1.3</v>
+        <v>-1.1</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>0</v>
@@ -3026,20 +3026,20 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Barrett Kent</t>
+          <t>Jhostin Betances</t>
         </is>
       </c>
       <c r="C18" s="4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>0.397</v>
+        <v>0.4</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.365</v>
+        <v>0.373</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>-1</v>
+        <v>-1.2</v>
       </c>
       <c r="G18" s="4" t="n">
         <v>0</v>
@@ -3317,20 +3317,20 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Wilner Berroteran</t>
+          <t>Sebastian Caseres</t>
         </is>
       </c>
       <c r="C11" s="4" t="n">
         <v>19</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.4</v>
+        <v>0.401</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.383</v>
+        <v>0.381</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>-1.4</v>
+        <v>-1.3</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>0</v>
@@ -3349,17 +3349,17 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Dioris De La Rosa</t>
+          <t>Anllelo Gutierrez</t>
         </is>
       </c>
       <c r="C12" s="4" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0.4</v>
+        <v>0.403</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0.378</v>
+        <v>0.381</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>-1.3</v>
@@ -3381,20 +3381,20 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Fabian Gallardo</t>
+          <t>Barrett Kent</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.4</v>
+        <v>0.397</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.378</v>
+        <v>0.365</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>-1.3</v>
+        <v>-1</v>
       </c>
       <c r="G13" s="4" t="n">
         <v>0</v>
@@ -3413,17 +3413,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Anderson Encarnacion</t>
+          <t>Wilner Berroteran</t>
         </is>
       </c>
       <c r="C14" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0.402</v>
+        <v>0.4</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.386</v>
+        <v>0.383</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>-1.4</v>
@@ -3445,20 +3445,20 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Jostin Alcantara</t>
+          <t>Fabian Gallardo</t>
         </is>
       </c>
       <c r="C15" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.399</v>
+        <v>0.4</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.394</v>
+        <v>0.378</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>-1.6</v>
+        <v>-1.3</v>
       </c>
       <c r="G15" s="4" t="n">
         <v>0</v>
@@ -3477,20 +3477,20 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Felix Tapia</t>
+          <t>Dioris De La Rosa</t>
         </is>
       </c>
       <c r="C16" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0.4</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.396</v>
+        <v>0.378</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>-1.7</v>
+        <v>-1.3</v>
       </c>
       <c r="G16" s="4" t="n">
         <v>0</v>
@@ -3509,7 +3509,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Steuri Amancio</t>
+          <t>Anderson Encarnacion</t>
         </is>
       </c>
       <c r="C17" s="4" t="n">
@@ -3519,10 +3519,10 @@
         <v>0.402</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.396</v>
+        <v>0.386</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>-1.7</v>
+        <v>-1.4</v>
       </c>
       <c r="G17" s="4" t="n">
         <v>0</v>
@@ -3539,26 +3539,36 @@
           <t>RP8</t>
         </is>
       </c>
-      <c r="B18" s="29" t="inlineStr">
-        <is>
-          <t>-- empty --</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="n"/>
-      <c r="D18" s="30" t="n"/>
-      <c r="E18" s="30" t="n"/>
-      <c r="F18" s="30" t="n"/>
-      <c r="G18" s="30" t="n"/>
-      <c r="H18" s="31" t="inlineStr">
-        <is>
-          <t>Sign FA</t>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Jostin Alcantara</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0.394</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Low leverage / depth</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>Total: 12 pitchers (target 13)</t>
+          <t>Total: 13 pitchers (target 13)</t>
         </is>
       </c>
     </row>
@@ -3655,20 +3665,20 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Elias Ledesma</t>
+          <t>Alex Gonzalez</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0.402</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.364</v>
+        <v>0.357</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>-2.9</v>
+        <v>-2.5</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>0</v>
@@ -3687,20 +3697,20 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Alexander Garcia</t>
+          <t>Elias Ledesma</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0.4</v>
+        <v>0.402</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.365</v>
+        <v>0.364</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>-3</v>
+        <v>-2.9</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0</v>
@@ -3719,20 +3729,20 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Johnny Slawinski</t>
+          <t>Alexander Garcia</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.399</v>
+        <v>0.4</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.354</v>
+        <v>0.365</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>-2.3</v>
+        <v>-3</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>0</v>
@@ -3751,20 +3761,20 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Luke LaCourse</t>
+          <t>Johnny Slawinski</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
         <v>20</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0.402</v>
+        <v>0.399</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.351</v>
+        <v>0.354</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>-2.1</v>
+        <v>-2.3</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0</v>
@@ -3783,20 +3793,20 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Jhon Almonte</t>
+          <t>Luke LaCourse</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
         <v>20</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.403</v>
+        <v>0.402</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.357</v>
+        <v>0.351</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>-2.5</v>
+        <v>-2.1</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>0</v>
@@ -3820,19 +3830,29 @@
           <t>RP1</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>-- empty --</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="n"/>
-      <c r="D11" s="30" t="n"/>
-      <c r="E11" s="30" t="n"/>
-      <c r="F11" s="30" t="n"/>
-      <c r="G11" s="30" t="n"/>
-      <c r="H11" s="31" t="inlineStr">
-        <is>
-          <t>Sign FA</t>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Felix Tapia</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Low leverage / depth</t>
         </is>
       </c>
     </row>
@@ -3842,19 +3862,29 @@
           <t>RP2</t>
         </is>
       </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>-- empty --</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="n"/>
-      <c r="D12" s="30" t="n"/>
-      <c r="E12" s="30" t="n"/>
-      <c r="F12" s="30" t="n"/>
-      <c r="G12" s="30" t="n"/>
-      <c r="H12" s="31" t="inlineStr">
-        <is>
-          <t>Sign FA</t>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Javier Rodriguez</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Low leverage / depth</t>
         </is>
       </c>
     </row>
@@ -3864,19 +3894,29 @@
           <t>RP3</t>
         </is>
       </c>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>-- empty --</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="n"/>
-      <c r="D13" s="30" t="n"/>
-      <c r="E13" s="30" t="n"/>
-      <c r="F13" s="30" t="n"/>
-      <c r="G13" s="30" t="n"/>
-      <c r="H13" s="31" t="inlineStr">
-        <is>
-          <t>Sign FA</t>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Steuri Amancio</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Low leverage / depth</t>
         </is>
       </c>
     </row>
@@ -3886,19 +3926,29 @@
           <t>RP4</t>
         </is>
       </c>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>-- empty --</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="n"/>
-      <c r="D14" s="30" t="n"/>
-      <c r="E14" s="30" t="n"/>
-      <c r="F14" s="30" t="n"/>
-      <c r="G14" s="30" t="n"/>
-      <c r="H14" s="31" t="inlineStr">
-        <is>
-          <t>Sign FA</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Steven Cabrera</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>0.401</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Low leverage / depth</t>
         </is>
       </c>
     </row>
@@ -3993,7 +4043,7 @@
     <row r="20">
       <c r="A20" s="20" t="inlineStr">
         <is>
-          <t>Total: 5 pitchers (target 13)</t>
+          <t>Total: 9 pitchers (target 13)</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5670,6 +5720,85 @@
         <v>-1.5</v>
       </c>
       <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Jacob Krieg</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Kauriel Leon</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Brayan Vergara</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="G22" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5779,7 +5908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5868,14 +5997,30 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Ryan Johnson</t>
+          <t>Rolando Anzola</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Flagged in flagged.txt — rerun once cleared</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Ryan Johnson</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Flagged in flagged.txt — rerun once cleared</t>
         </is>
@@ -14911,27 +15056,27 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Walbert Urena</t>
+          <t>Jack Kochanowicz</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.334</v>
+        <v>0.327</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.312</v>
+        <v>0.325</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.4</v>
+        <v>-0.4</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Back-end starter</t>
+          <t>Innings eater</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
60/40 fld-to-bat weighting for Utility IF / OF roles
Was: (positions, fld_sum, wOBA_tiebreak) — bat only mattered as a
hard tiebreak when both positions count and fielding sum tied.

Now: (positions, 0.6*fld_sum + 0.4*bat_war) — multi-position is still
a hard prerequisite of utility (more positions wins outright), but
within a tied position count the weighted glove+bat score lets a
slightly-worse-glove player with a meaningfully better bat overtake
a glove-only specialist. Both terms are in WAR units so the 60/40
split is on like-for-like (war_hitting is the calibrated bat-WAR,
not raw wOBA).

Bench refinement's UTIL_ROLE_FNS uses the same shape — refinement
swaps and classify_bench's role-picker now agree on what "best
utility" means.

Spot-check (AZ): Luis Urias (fld +6.47, bat -0.60) lands MLB Util IF,
Jorge Barrosa (fld +9.55, bat -1.10) keeps MLB Util OF. Lower levels
similarly weight bat into picks.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/LAA_roster_system.xlsx
+++ b/outputs/LAA_roster_system.xlsx
@@ -818,10 +818,10 @@
         </is>
       </c>
       <c r="E8" s="4" t="n">
-        <v>-3.92</v>
+        <v>-4.13</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.52</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="9">
@@ -842,10 +842,10 @@
         </is>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-5.53</v>
+        <v>-5.35</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>-0.57</v>
+        <v>-0.27</v>
       </c>
     </row>
     <row r="10">
@@ -12387,11 +12387,11 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Alexander Rincon</t>
+          <t>Samil Dishmey</t>
         </is>
       </c>
       <c r="C45" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
@@ -12399,16 +12399,16 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>0.202</v>
+        <v>0.207</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>0.287</v>
+        <v>0.263</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.056</v>
       </c>
       <c r="H45" s="4" t="n">
-        <v>1.82</v>
+        <v>-2.72</v>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
@@ -12798,11 +12798,11 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Samil Dishmey</t>
+          <t>Alexander Rincon</t>
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
@@ -12810,16 +12810,16 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.207</v>
+        <v>0.202</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.263</v>
+        <v>0.287</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>0.056</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>-2.72</v>
+        <v>1.82</v>
       </c>
       <c r="I13" s="4" t="inlineStr"/>
     </row>
@@ -13128,20 +13128,20 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Samil Dishmey</t>
+          <t>Alexander Rincon</t>
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>0.196</v>
+        <v>0.212</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0.207</v>
+        <v>0.202</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>-0.011</v>
+        <v>0.01</v>
       </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
@@ -13149,7 +13149,7 @@
     <row r="25">
       <c r="A25" s="20" t="inlineStr">
         <is>
-          <t>Est. R/G: 0.23</t>
+          <t>Est. R/G: 0.29</t>
         </is>
       </c>
     </row>
@@ -13205,7 +13205,7 @@
     </row>
     <row r="28">
       <c r="A28" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
@@ -13234,7 +13234,7 @@
     </row>
     <row r="29">
       <c r="A29" s="18" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
@@ -13243,31 +13243,27 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Samil Dishmey</t>
+          <t>Sandy Ruiz</t>
         </is>
       </c>
       <c r="D29" s="4" t="n">
         <v>21</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>0.234</v>
+        <v>0.185</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>0.207</v>
+        <v>0.185</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0.026</v>
+        <v>0</v>
       </c>
       <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>swap from Sandy Ruiz</t>
-        </is>
-      </c>
+      <c r="I29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="18" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B30" s="18" t="inlineStr">
         <is>
@@ -13296,7 +13292,7 @@
     </row>
     <row r="31">
       <c r="A31" s="18" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
@@ -13325,7 +13321,7 @@
     </row>
     <row r="32">
       <c r="A32" s="18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B32" s="18" t="inlineStr">
         <is>
@@ -13354,7 +13350,7 @@
     </row>
     <row r="33">
       <c r="A33" s="18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
@@ -13383,7 +13379,7 @@
     </row>
     <row r="34">
       <c r="A34" s="18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
@@ -13412,7 +13408,7 @@
     </row>
     <row r="35">
       <c r="A35" s="18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
@@ -13441,7 +13437,7 @@
     </row>
     <row r="36">
       <c r="A36" s="18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
@@ -13468,14 +13464,14 @@
       <c r="H36" s="4" t="n"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>swap from Samil Dishmey</t>
+          <t>swap from Alexander Rincon</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="20" t="inlineStr">
         <is>
-          <t>Est. R/G: 0.66</t>
+          <t>Est. R/G: 0.47</t>
         </is>
       </c>
     </row>

</xml_diff>